<commit_message>
Add cleaned notebook and all updated figures
</commit_message>
<xml_diff>
--- a/tables/classification_report.xlsx
+++ b/tables/classification_report.xlsx
@@ -465,13 +465,13 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.998218421521468</v>
+        <v>0.9986666666666667</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9991084165477889</v>
+        <v>0.9993328885923949</v>
       </c>
       <c r="E2" t="n">
-        <v>5613</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="3">
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9881855052019044</v>
+        <v>0.9624177346726706</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9343114371457152</v>
+        <v>0.9261666666666667</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9604936155626017</v>
+        <v>0.9439442840156277</v>
       </c>
       <c r="E3" t="n">
-        <v>5998</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="4">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9987339482727438</v>
+        <v>0.998970310622962</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9691119691119691</v>
+        <v>0.9701666666666666</v>
       </c>
       <c r="D4" t="n">
-        <v>0.983700008907099</v>
+        <v>0.9843578253149573</v>
       </c>
       <c r="E4" t="n">
-        <v>5698</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="5">
@@ -519,16 +519,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9557239057239058</v>
+        <v>0.9418411432369558</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9479044915678745</v>
+        <v>0.9449816605535178</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9517981389890183</v>
+        <v>0.9434087882822902</v>
       </c>
       <c r="E5" t="n">
-        <v>5989</v>
+        <v>5998</v>
       </c>
     </row>
     <row r="6">
@@ -538,16 +538,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.2430213464696223</v>
+        <v>0.246353322528363</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9487179487179487</v>
+        <v>0.9712460063897763</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3869281045751634</v>
+        <v>0.3930187459599224</v>
       </c>
       <c r="E6" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="7">
@@ -557,16 +557,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9929038430872269</v>
+        <v>0.9930321255684319</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9873929590865842</v>
+        <v>0.9855146309506478</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9901407330842014</v>
+        <v>0.9892590968873302</v>
       </c>
       <c r="E7" t="n">
-        <v>12612</v>
+        <v>13738</v>
       </c>
     </row>
     <row r="8">
@@ -576,16 +576,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9964218776622934</v>
+        <v>0.9952710690761696</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9813727135425407</v>
+        <v>0.9821666666666666</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9888400405816706</v>
+        <v>0.9886754466907138</v>
       </c>
       <c r="E8" t="n">
-        <v>5959</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="9">
@@ -595,13 +595,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.9923664122137404</v>
+        <v>0.9941520467836257</v>
       </c>
       <c r="C9" t="n">
         <v>0.9997738068310337</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9960563380281691</v>
+        <v>0.9969550016916657</v>
       </c>
       <c r="E9" t="n">
         <v>4421</v>
@@ -614,13 +614,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9859341386728446</v>
+        <v>0.9917743830787309</v>
       </c>
       <c r="C10" t="n">
-        <v>0.993</v>
+        <v>0.9846666666666667</v>
       </c>
       <c r="D10" t="n">
-        <v>0.989454454870049</v>
+        <v>0.988207744417496</v>
       </c>
       <c r="E10" t="n">
         <v>6000</v>
@@ -633,16 +633,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.9548432381843707</v>
+        <v>0.9742368095994354</v>
       </c>
       <c r="C11" t="n">
-        <v>0.8987007267121779</v>
+        <v>0.9201666666666667</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9259217243335224</v>
+        <v>0.9464301019970858</v>
       </c>
       <c r="E11" t="n">
-        <v>4541</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="12">
@@ -652,16 +652,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.9705825735435661</v>
+        <v>0.9694559285596164</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9705825735435661</v>
+        <v>0.9694559285596164</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9705825735435661</v>
+        <v>0.9694559285596164</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9705825735435661</v>
+        <v>0.9694559285596164</v>
       </c>
     </row>
     <row r="13">
@@ -671,16 +671,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.9108134215488652</v>
+        <v>0.9098048945167345</v>
       </c>
       <c r="C13" t="n">
-        <v>0.9658504474237313</v>
+        <v>0.9683516104724976</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9172441575479283</v>
+        <v>0.9173589923849483</v>
       </c>
       <c r="E13" t="n">
-        <v>57143</v>
+        <v>60470</v>
       </c>
     </row>
     <row r="14">
@@ -690,16 +690,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.9822647909975512</v>
+        <v>0.9806468521461216</v>
       </c>
       <c r="C14" t="n">
-        <v>0.9705825735435661</v>
+        <v>0.9694559285596164</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9751020177333712</v>
+        <v>0.9737927908266789</v>
       </c>
       <c r="E14" t="n">
-        <v>57143</v>
+        <v>60470</v>
       </c>
     </row>
   </sheetData>

</xml_diff>